<commit_message>
add northwind data and columns
</commit_message>
<xml_diff>
--- a/week 09/NorthwindTablesAndColumns.xlsx
+++ b/week 09/NorthwindTablesAndColumns.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alondramartinez\Documents\DataAnalytics\week 09\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1D40BFF2-531D-4BFD-AE95-8ABD7DDE25D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F326F18D-05EE-41D3-B6C4-660AC2B42225}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2295" yWindow="2295" windowWidth="28800" windowHeight="15285" xr2:uid="{901F5D27-877F-4C94-89AE-9A9B6ECE5CB6}"/>
+    <workbookView xWindow="14040" yWindow="2895" windowWidth="14760" windowHeight="12585" xr2:uid="{901F5D27-877F-4C94-89AE-9A9B6ECE5CB6}"/>
   </bookViews>
   <sheets>
     <sheet name="Northwind Columns" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="124">
   <si>
     <t>table_name</t>
   </si>
@@ -308,6 +308,105 @@
   </si>
   <si>
     <t>New Column Name?</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>mo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes </t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> yes </t>
+  </si>
+  <si>
+    <t>currency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes   </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> no</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">product </t>
+  </si>
+  <si>
+    <t xml:space="preserve">order date </t>
+  </si>
+  <si>
+    <t>category name</t>
+  </si>
+  <si>
+    <t>customer ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">company name </t>
+  </si>
+  <si>
+    <t>contact name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact title </t>
+  </si>
+  <si>
+    <t>employee ID</t>
+  </si>
+  <si>
+    <t>last name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">first name </t>
+  </si>
+  <si>
+    <t xml:space="preserve">title of courtesy </t>
+  </si>
+  <si>
+    <t>birth date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hire date </t>
+  </si>
+  <si>
+    <t>postal code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">home phone </t>
+  </si>
+  <si>
+    <t xml:space="preserve">employee ID </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Territory ID </t>
+  </si>
+  <si>
+    <t>Order ID</t>
+  </si>
+  <si>
+    <t>Employee ID</t>
+  </si>
+  <si>
+    <t>0 22</t>
   </si>
 </sst>
 </file>
@@ -706,8 +805,8 @@
     <col min="9" max="9" width="19.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="26" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.5703125" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" customWidth="1"/>
+    <col min="12" max="12" width="23.85546875" customWidth="1"/>
+    <col min="13" max="13" width="19" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -756,7 +855,7 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>5</v>
+        <v>123</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
@@ -770,6 +869,22 @@
       <c r="E2" s="1">
         <v>4</v>
       </c>
+      <c r="F2" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H2" t="s">
+        <v>91</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -787,6 +902,24 @@
       <c r="E3" s="1">
         <v>30</v>
       </c>
+      <c r="F3" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -804,6 +937,24 @@
       <c r="E4" s="1">
         <v>16</v>
       </c>
+      <c r="F4" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -821,6 +972,24 @@
       <c r="E5" s="1">
         <v>16</v>
       </c>
+      <c r="F5" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -838,6 +1007,24 @@
       <c r="E6" s="2">
         <v>10</v>
       </c>
+      <c r="F6" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
@@ -855,6 +1042,24 @@
       <c r="E7" s="2">
         <v>80</v>
       </c>
+      <c r="F7" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
@@ -872,6 +1077,22 @@
       <c r="E8" s="2">
         <v>60</v>
       </c>
+      <c r="F8" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
@@ -889,6 +1110,24 @@
       <c r="E9" s="2">
         <v>60</v>
       </c>
+      <c r="F9" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
@@ -906,6 +1145,22 @@
       <c r="E10" s="2">
         <v>120</v>
       </c>
+      <c r="F10" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
@@ -923,6 +1178,24 @@
       <c r="E11" s="2">
         <v>30</v>
       </c>
+      <c r="F11" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
@@ -940,13 +1213,31 @@
       <c r="E12" s="2">
         <v>30</v>
       </c>
+      <c r="F12" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>16</v>
+        <v>94</v>
       </c>
       <c r="B13" s="2">
-        <v>8</v>
+        <v>33</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>23</v>
@@ -956,6 +1247,24 @@
       </c>
       <c r="E13" s="2">
         <v>20</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
@@ -974,6 +1283,24 @@
       <c r="E14" s="2">
         <v>30</v>
       </c>
+      <c r="F14" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
@@ -991,6 +1318,24 @@
       <c r="E15" s="2">
         <v>48</v>
       </c>
+      <c r="F15" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
@@ -1008,8 +1353,26 @@
       <c r="E16" s="2">
         <v>48</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F16" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>27</v>
       </c>
@@ -1025,8 +1388,26 @@
       <c r="E17" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F17" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>27</v>
       </c>
@@ -1042,8 +1423,22 @@
       <c r="E18" s="1">
         <v>40</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>27</v>
       </c>
@@ -1059,8 +1454,26 @@
       <c r="E19" s="1">
         <v>20</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F19" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>27</v>
       </c>
@@ -1076,8 +1489,26 @@
       <c r="E20" s="1">
         <v>60</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F20" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>27</v>
       </c>
@@ -1093,8 +1524,26 @@
       <c r="E21" s="1">
         <v>50</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F21" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>27</v>
       </c>
@@ -1110,8 +1559,26 @@
       <c r="E22" s="1">
         <v>8</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F22" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>27</v>
       </c>
@@ -1127,8 +1594,26 @@
       <c r="E23" s="1">
         <v>8</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F23" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>27</v>
       </c>
@@ -1144,8 +1629,26 @@
       <c r="E24" s="1">
         <v>120</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F24" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>27</v>
       </c>
@@ -1161,8 +1664,26 @@
       <c r="E25" s="1">
         <v>30</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F25" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>27</v>
       </c>
@@ -1178,8 +1699,26 @@
       <c r="E26" s="1">
         <v>30</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F26" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>27</v>
       </c>
@@ -1195,8 +1734,26 @@
       <c r="E27" s="1">
         <v>20</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F27" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>27</v>
       </c>
@@ -1212,8 +1769,26 @@
       <c r="E28" s="1">
         <v>30</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F28" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
@@ -1229,8 +1804,26 @@
       <c r="E29" s="1">
         <v>48</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F29" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K29" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>27</v>
       </c>
@@ -1246,8 +1839,26 @@
       <c r="E30" s="1">
         <v>8</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F30" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>27</v>
       </c>
@@ -1263,8 +1874,26 @@
       <c r="E31" s="1">
         <v>16</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F31" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>27</v>
       </c>
@@ -1280,8 +1909,26 @@
       <c r="E32" s="1">
         <v>16</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F32" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>27</v>
       </c>
@@ -1297,8 +1944,26 @@
       <c r="E33" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F33" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K33" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>27</v>
       </c>
@@ -1314,8 +1979,26 @@
       <c r="E34" s="1">
         <v>510</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F34" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J34" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K34" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>42</v>
       </c>
@@ -1331,8 +2014,26 @@
       <c r="E35" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F35" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K35" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>42</v>
       </c>
@@ -1348,8 +2049,26 @@
       <c r="E36" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F36" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K36" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>44</v>
       </c>
@@ -1365,8 +2084,26 @@
       <c r="E37" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F37" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K37" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>44</v>
       </c>
@@ -1382,8 +2119,26 @@
       <c r="E38" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F38" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J38" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K38" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>44</v>
       </c>
@@ -1399,8 +2154,26 @@
       <c r="E39" s="1">
         <v>8</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F39" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H39" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I39" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J39" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K39" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>44</v>
       </c>
@@ -1416,8 +2189,26 @@
       <c r="E40" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F40" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I40" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J40" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K40" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>44</v>
       </c>
@@ -1433,8 +2224,26 @@
       <c r="E41" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F41" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I41" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J41" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K41" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>53</v>
       </c>
@@ -1450,8 +2259,26 @@
       <c r="E42" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F42" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H42" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="J42" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K42" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>53</v>
       </c>
@@ -1467,8 +2294,29 @@
       <c r="E43" s="2">
         <v>10</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F43" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H43" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I43" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="J43" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K43" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="L43" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>53</v>
       </c>
@@ -1484,8 +2332,29 @@
       <c r="E44" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F44" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="H44" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="J44" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K44" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="L44" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>53</v>
       </c>
@@ -1501,8 +2370,26 @@
       <c r="E45" s="2">
         <v>8</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F45" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H45" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I45" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="J45" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K45" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>53</v>
       </c>
@@ -1518,8 +2405,26 @@
       <c r="E46" s="2">
         <v>8</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F46" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H46" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I46" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J46" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K46" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>53</v>
       </c>
@@ -1535,8 +2440,26 @@
       <c r="E47" s="2">
         <v>8</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F47" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="H47" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I47" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J47" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K47" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>53</v>
       </c>
@@ -1552,8 +2475,26 @@
       <c r="E48" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F48" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="H48" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I48" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J48" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K48" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>53</v>
       </c>
@@ -1569,8 +2510,26 @@
       <c r="E49" s="2">
         <v>8</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F49" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="H49" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I49" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J49" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K49" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>53</v>
       </c>
@@ -1586,8 +2545,26 @@
       <c r="E50" s="2">
         <v>80</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F50" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H50" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="I50" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J50" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K50" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>53</v>
       </c>
@@ -1603,8 +2580,26 @@
       <c r="E51" s="2">
         <v>120</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F51" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H51" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I51" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J51" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K51" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>53</v>
       </c>
@@ -1620,8 +2615,26 @@
       <c r="E52" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F52" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I52" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J52" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K52" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>53</v>
       </c>
@@ -1637,8 +2650,26 @@
       <c r="E53" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F53" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H53" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I53" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J53" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K53" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>53</v>
       </c>
@@ -1654,8 +2685,26 @@
       <c r="E54" s="2">
         <v>20</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F54" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I54" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J54" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K54" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>53</v>
       </c>
@@ -1671,8 +2720,26 @@
       <c r="E55" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F55" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H55" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I55" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J55" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K55" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>65</v>
       </c>
@@ -1688,8 +2755,26 @@
       <c r="E56" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F56" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I56" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J56" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K56" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>65</v>
       </c>
@@ -1705,8 +2790,26 @@
       <c r="E57" s="1">
         <v>80</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F57" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H57" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I57" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="J57" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K57" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>65</v>
       </c>
@@ -1722,8 +2825,26 @@
       <c r="E58" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F58" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="H58" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I58" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J58" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="K58" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>65</v>
       </c>
@@ -1739,8 +2860,26 @@
       <c r="E59" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F59" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I59" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J59" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K59" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>65</v>
       </c>
@@ -1756,8 +2895,26 @@
       <c r="E60" s="1">
         <v>40</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F60" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H60" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I60" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J60" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K60" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>65</v>
       </c>
@@ -1773,8 +2930,29 @@
       <c r="E61" s="1">
         <v>8</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F61" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H61" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I61" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J61" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K61" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="L61" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>65</v>
       </c>
@@ -1790,8 +2968,29 @@
       <c r="E62" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F62" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G62" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H62" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I62" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J62" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="K62" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L62" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>65</v>
       </c>
@@ -1807,8 +3006,29 @@
       <c r="E63" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F63" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G63" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H63" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I63" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J63" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="K63" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="L63" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>65</v>
       </c>
@@ -1824,8 +3044,29 @@
       <c r="E64" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F64" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G64" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H64" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I64" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J64" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="K64" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="L64" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>65</v>
       </c>
@@ -1841,8 +3082,26 @@
       <c r="E65" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F65" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H65" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="I65" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J65" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K65" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>22</v>
       </c>
@@ -1858,8 +3117,29 @@
       <c r="E66" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F66" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H66" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I66" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J66" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K66" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="L66" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>22</v>
       </c>
@@ -1875,8 +3155,26 @@
       <c r="E67" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F67" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H67" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J67" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K67" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>76</v>
       </c>
@@ -1892,8 +3190,26 @@
       <c r="E68" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F68" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="H68" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I68" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J68" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K68" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>76</v>
       </c>
@@ -1909,8 +3225,26 @@
       <c r="E69" s="1">
         <v>80</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F69" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="H69" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I69" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J69" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K69" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>76</v>
       </c>
@@ -1926,8 +3260,29 @@
       <c r="E70" s="1">
         <v>48</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F70" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H70" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="J70" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K70" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="L70" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>78</v>
       </c>
@@ -1943,8 +3298,29 @@
       <c r="E71" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F71" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H71" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I71" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J71" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K71" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="L71" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>78</v>
       </c>
@@ -1960,8 +3336,29 @@
       <c r="E72" s="2">
         <v>80</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F72" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H72" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="I72" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J72" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K72" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="L72" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>78</v>
       </c>
@@ -1977,8 +3374,29 @@
       <c r="E73" s="2">
         <v>60</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F73" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H73" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I73" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J73" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K73" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="L73" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>78</v>
       </c>
@@ -1994,8 +3412,29 @@
       <c r="E74" s="2">
         <v>60</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F74" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H74" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I74" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J74" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K74" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="L74" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>78</v>
       </c>
@@ -2011,8 +3450,29 @@
       <c r="E75" s="2">
         <v>120</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F75" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H75" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="I75" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J75" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K75" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="L75" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>78</v>
       </c>
@@ -2028,8 +3488,29 @@
       <c r="E76" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F76" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H76" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I76" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J76" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K76" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="L76" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>78</v>
       </c>
@@ -2045,8 +3526,29 @@
       <c r="E77" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F77" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H77" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I77" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J77" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K77" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="L77" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>78</v>
       </c>
@@ -2062,8 +3564,29 @@
       <c r="E78" s="2">
         <v>20</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F78" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G78" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H78" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I78" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J78" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K78" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="L78" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>78</v>
       </c>
@@ -2079,8 +3602,29 @@
       <c r="E79" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F79" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H79" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I79" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J79" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K79" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="L79" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>78</v>
       </c>
@@ -2096,8 +3640,29 @@
       <c r="E80" s="2">
         <v>48</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F80" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G80" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H80" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I80" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J80" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K80" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="L80" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>78</v>
       </c>
@@ -2113,8 +3678,29 @@
       <c r="E81" s="2">
         <v>48</v>
       </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F81" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H81" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I81" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J81" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K81" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="L81" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>78</v>
       </c>
@@ -2130,8 +3716,29 @@
       <c r="E82" s="2">
         <v>16</v>
       </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F82" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G82" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H82" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I82" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J82" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K82" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="L82" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>80</v>
       </c>
@@ -2147,8 +3754,26 @@
       <c r="E83" s="1">
         <v>40</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F83" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="H83" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="I83" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J83" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K83" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>80</v>
       </c>
@@ -2164,8 +3789,26 @@
       <c r="E84" s="1">
         <v>100</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F84" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G84" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H84" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I84" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J84" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K84" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>80</v>
       </c>
@@ -2180,6 +3823,24 @@
       </c>
       <c r="E85" s="1">
         <v>4</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H85" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I85" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="J85" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K85" s="1" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -2188,6 +3849,25 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ced60a7f-99b1-48d2-b555-34851c8026ae" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9e0b35a9-e6cb-436b-81d4-4440ba439ca5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <SharedWithUsers xmlns="ced60a7f-99b1-48d2-b555-34851c8026ae">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <MediaLengthInSeconds xmlns="9e0b35a9-e6cb-436b-81d4-4440ba439ca5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CA5D0A6329BB324E86983B32928CFC2E" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d7eac4bce3bbb09c82bd908806be82e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9e0b35a9-e6cb-436b-81d4-4440ba439ca5" xmlns:ns3="ced60a7f-99b1-48d2-b555-34851c8026ae" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eb51570e5b7cb8bd524bc2df5324d4a3" ns2:_="" ns3:_="">
     <xsd:import namespace="9e0b35a9-e6cb-436b-81d4-4440ba439ca5"/>
@@ -2428,25 +4108,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ced60a7f-99b1-48d2-b555-34851c8026ae" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9e0b35a9-e6cb-436b-81d4-4440ba439ca5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <SharedWithUsers xmlns="ced60a7f-99b1-48d2-b555-34851c8026ae">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <MediaLengthInSeconds xmlns="9e0b35a9-e6cb-436b-81d4-4440ba439ca5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2457,6 +4118,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BB560F9-4CC1-4243-8F16-7FDC2CD703FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ced60a7f-99b1-48d2-b555-34851c8026ae"/>
+    <ds:schemaRef ds:uri="9e0b35a9-e6cb-436b-81d4-4440ba439ca5"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA285021-94D7-4152-B2E7-B2D9504C2DBD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2475,17 +4147,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2BB560F9-4CC1-4243-8F16-7FDC2CD703FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ced60a7f-99b1-48d2-b555-34851c8026ae"/>
-    <ds:schemaRef ds:uri="9e0b35a9-e6cb-436b-81d4-4440ba439ca5"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0257D61C-6042-483B-9C34-3DE0D82CB154}">
   <ds:schemaRefs>

</xml_diff>